<commit_message>
Change python version to 4.11 for better compatibility
Signed-off-by: Paul Ammann <p.ammann@campus.tu-berlin.de>
</commit_message>
<xml_diff>
--- a/Deliverables/sprint-01/Bill_of_Materials.xlsx
+++ b/Deliverables/sprint-01/Bill_of_Materials.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Paul\Documents\Uni\SS26\AMOS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Paul\Documents\Arbeit\DEV\amos2026ss02-automated-thematic-analysis\Deliverables\sprint-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF2257E7-8863-499F-A056-121A8805A0E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C175AE1E-1A7C-437A-9EFF-B26EAE57B2B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3758C20-B850-4BD9-899F-233016B9C0F5}"/>
   </bookViews>
@@ -816,7 +816,7 @@
         <v>70</v>
       </c>
       <c r="D4" s="2">
-        <v>3.14</v>
+        <v>3.11</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>69</v>

</xml_diff>